<commit_message>
update paper analysis and CoT
</commit_message>
<xml_diff>
--- a/analysis/dataview/paper.xlsx
+++ b/analysis/dataview/paper.xlsx
@@ -9,16 +9,17 @@
   <sheets>
     <sheet name="Unique Variants" sheetId="1" r:id="rId1"/>
     <sheet name="SubTask" sheetId="2" r:id="rId2"/>
-    <sheet name="ModelFamily" sheetId="3" r:id="rId3"/>
-    <sheet name="ModelName" sheetId="4" r:id="rId4"/>
-    <sheet name="Mode" sheetId="5" r:id="rId5"/>
+    <sheet name="ExampleType" sheetId="3" r:id="rId3"/>
+    <sheet name="ModelFamily" sheetId="4" r:id="rId4"/>
+    <sheet name="ModelName" sheetId="5" r:id="rId5"/>
+    <sheet name="Mode" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="47">
   <si>
     <t>Unique Variants</t>
   </si>
@@ -56,6 +57,15 @@
     <t>outline_extraction</t>
   </si>
   <si>
+    <t>FewShot</t>
+  </si>
+  <si>
+    <t>OneShot</t>
+  </si>
+  <si>
+    <t>ZeroShot</t>
+  </si>
+  <si>
     <t>max</t>
   </si>
   <si>
@@ -113,7 +123,16 @@
     <t>Phi-3.5-mini-instruct</t>
   </si>
   <si>
+    <t>Qwen2.5-0.5B-Instruct</t>
+  </si>
+  <si>
+    <t>Qwen2.5-1.5B-Instruct</t>
+  </si>
+  <si>
     <t>Qwen2.5-32B-Instruct</t>
+  </si>
+  <si>
+    <t>Qwen2.5-3B-Instruct</t>
   </si>
   <si>
     <t>Qwen2.5-72B-Instruct</t>
@@ -519,7 +538,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -535,7 +554,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -575,13 +594,13 @@
         <v>9</v>
       </c>
       <c r="B2">
-        <v>13.6571875</v>
+        <v>13.68684210526316</v>
       </c>
       <c r="C2">
-        <v>7.458812166253526</v>
+        <v>7.017452800855399</v>
       </c>
       <c r="D2">
-        <v>32</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -589,13 +608,13 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>13.96625</v>
+        <v>12.82157894736842</v>
       </c>
       <c r="C3">
-        <v>11.08050067286178</v>
+        <v>10.64656765558507</v>
       </c>
       <c r="D3">
-        <v>32</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -603,13 +622,13 @@
         <v>11</v>
       </c>
       <c r="B4">
-        <v>47.13161290322581</v>
+        <v>46.1927027027027</v>
       </c>
       <c r="C4">
-        <v>31.25184848898533</v>
+        <v>30.9379196176839</v>
       </c>
       <c r="D4">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -619,224 +638,63 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
       <c r="B1" s="1" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="1">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="B2">
+        <v>4.581666666666666</v>
+      </c>
+      <c r="C2">
+        <v>2.823362652346784</v>
+      </c>
+      <c r="D2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C2">
-        <v>10.26833333333333</v>
-      </c>
-      <c r="D2">
-        <v>6.92675224522046</v>
-      </c>
-      <c r="E2">
-        <v>6</v>
-      </c>
-      <c r="F2">
-        <v>10.26833333333333</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="1">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="B3">
+        <v>5.116666666666666</v>
+      </c>
+      <c r="C3">
+        <v>3.303874493177165</v>
+      </c>
+      <c r="D3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C3">
-        <v>33.00777777777778</v>
-      </c>
-      <c r="D3">
-        <v>29.88116769817632</v>
-      </c>
-      <c r="E3">
-        <v>18</v>
-      </c>
-      <c r="F3">
-        <v>42.07833333333333</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" s="1">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
+      <c r="B4">
+        <v>3.983333333333334</v>
       </c>
       <c r="C4">
-        <v>37.60333333333333</v>
+        <v>3.994389398477153</v>
       </c>
       <c r="D4">
-        <v>18.19036961325049</v>
-      </c>
-      <c r="E4">
-        <v>6</v>
-      </c>
-      <c r="F4">
-        <v>37.60333333333333</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="1">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>5</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="1">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6">
-        <v>42.98499999999999</v>
-      </c>
-      <c r="D6">
-        <v>41.07003420987132</v>
-      </c>
-      <c r="E6">
-        <v>6</v>
-      </c>
-      <c r="F6">
-        <v>42.98499999999999</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="1">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7">
-        <v>6.235</v>
-      </c>
-      <c r="D7">
-        <v>6.190126816148438</v>
-      </c>
-      <c r="E7">
-        <v>6</v>
-      </c>
-      <c r="F7">
-        <v>6.235</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" s="1">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8">
-        <v>23.55233333333333</v>
-      </c>
-      <c r="D8">
-        <v>19.64752940217155</v>
-      </c>
-      <c r="E8">
-        <v>30</v>
-      </c>
-      <c r="F8">
-        <v>43.70666666666667</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="1">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9">
-        <v>11.51</v>
-      </c>
-      <c r="D9">
-        <v>7.301079372257227</v>
-      </c>
-      <c r="E9">
-        <v>6</v>
-      </c>
-      <c r="F9">
-        <v>11.51</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" s="1">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10">
-        <v>27.10166666666667</v>
-      </c>
-      <c r="D10">
-        <v>22.22504210719671</v>
-      </c>
-      <c r="E10">
-        <v>6</v>
-      </c>
-      <c r="F10">
-        <v>27.10166666666667</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" s="1">
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11">
-        <v>38.35</v>
-      </c>
-      <c r="D11">
-        <v>33.34598806453334</v>
-      </c>
-      <c r="E11">
-        <v>6</v>
-      </c>
-      <c r="F11">
-        <v>38.35</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -846,245 +704,224 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6">
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="1">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2">
+        <v>10.26833333333333</v>
+      </c>
+      <c r="D2">
+        <v>6.92675224522046</v>
+      </c>
+      <c r="E2">
+        <v>6</v>
+      </c>
+      <c r="F2">
+        <v>10.26833333333333</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="1">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3">
+        <v>26.82111111111111</v>
+      </c>
+      <c r="D3">
+        <v>27.13810065759185</v>
+      </c>
+      <c r="E3">
+        <v>36</v>
+      </c>
+      <c r="F3">
+        <v>42.07833333333333</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="1">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4">
+        <v>37.60333333333333</v>
+      </c>
+      <c r="D4">
+        <v>18.19036961325049</v>
+      </c>
+      <c r="E4">
+        <v>6</v>
+      </c>
+      <c r="F4">
+        <v>37.60333333333333</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="1">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6">
+        <v>42.98499999999999</v>
+      </c>
+      <c r="D6">
+        <v>41.07003420987132</v>
+      </c>
+      <c r="E6">
+        <v>6</v>
+      </c>
+      <c r="F6">
+        <v>42.98499999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="1">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7">
+        <v>6.235</v>
+      </c>
+      <c r="D7">
+        <v>6.190126816148438</v>
+      </c>
+      <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7">
+        <v>6.235</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="1">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8">
+        <v>23.55233333333333</v>
+      </c>
+      <c r="D8">
+        <v>19.64752940217155</v>
+      </c>
+      <c r="E8">
+        <v>30</v>
+      </c>
+      <c r="F8">
+        <v>43.70666666666667</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9">
+        <v>11.51</v>
+      </c>
+      <c r="D9">
+        <v>7.301079372257227</v>
+      </c>
+      <c r="E9">
+        <v>6</v>
+      </c>
+      <c r="F9">
+        <v>11.51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="1">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="1" t="s">
+      <c r="B10" t="s">
         <v>24</v>
       </c>
-      <c r="B3">
-        <v>16.45833333333333</v>
-      </c>
-      <c r="C3">
-        <v>4.190720304036844</v>
-      </c>
-      <c r="D3">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="1" t="s">
+      <c r="C10">
+        <v>27.10166666666667</v>
+      </c>
+      <c r="D10">
+        <v>22.22504210719671</v>
+      </c>
+      <c r="E10">
+        <v>6</v>
+      </c>
+      <c r="F10">
+        <v>27.10166666666667</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="1">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
         <v>25</v>
       </c>
-      <c r="B4">
-        <v>43.70666666666667</v>
-      </c>
-      <c r="C4">
-        <v>31.03935351560445</v>
-      </c>
-      <c r="D4">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5">
-        <v>13.29833333333333</v>
-      </c>
-      <c r="C5">
-        <v>10.07747670137057</v>
-      </c>
-      <c r="D5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6">
-        <v>28.06666666666667</v>
-      </c>
-      <c r="C6">
-        <v>18.28862998331659</v>
-      </c>
-      <c r="D6">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7">
-        <v>16.23166666666667</v>
-      </c>
-      <c r="C7">
-        <v>7.690826786936935</v>
-      </c>
-      <c r="D7">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8">
-        <v>27.10166666666667</v>
-      </c>
-      <c r="C8">
-        <v>22.22504210719671</v>
-      </c>
-      <c r="D8">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9">
-        <v>11.51</v>
-      </c>
-      <c r="C9">
-        <v>7.301079372257227</v>
-      </c>
-      <c r="D9">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10">
-        <v>17.22166666666667</v>
-      </c>
-      <c r="C10">
-        <v>15.55391322679494</v>
-      </c>
-      <c r="D10">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11">
-        <v>39.72333333333334</v>
-      </c>
       <c r="C11">
-        <v>35.28562351251097</v>
+        <v>38.35</v>
       </c>
       <c r="D11">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12">
-        <v>42.07833333333333</v>
-      </c>
-      <c r="C12">
-        <v>33.11973455006346</v>
-      </c>
-      <c r="D12">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13">
-        <v>10.26833333333333</v>
-      </c>
-      <c r="C13">
-        <v>6.92675224522046</v>
-      </c>
-      <c r="D13">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14">
-        <v>42.98499999999999</v>
-      </c>
-      <c r="C14">
-        <v>41.07003420987132</v>
-      </c>
-      <c r="D14">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15">
-        <v>37.60333333333333</v>
-      </c>
-      <c r="C15">
-        <v>18.19036961325049</v>
-      </c>
-      <c r="D15">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B16">
+        <v>33.34598806453334</v>
+      </c>
+      <c r="E11">
+        <v>6</v>
+      </c>
+      <c r="F11">
         <v>38.35</v>
-      </c>
-      <c r="C16">
-        <v>33.34598806453334</v>
-      </c>
-      <c r="D16">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B17">
-        <v>6.235</v>
-      </c>
-      <c r="C17">
-        <v>6.190126816148438</v>
-      </c>
-      <c r="D17">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1094,6 +931,296 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3">
+        <v>16.45833333333333</v>
+      </c>
+      <c r="C3">
+        <v>4.190720304036844</v>
+      </c>
+      <c r="D3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4">
+        <v>43.70666666666667</v>
+      </c>
+      <c r="C4">
+        <v>31.03935351560445</v>
+      </c>
+      <c r="D4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5">
+        <v>13.29833333333333</v>
+      </c>
+      <c r="C5">
+        <v>10.07747670137057</v>
+      </c>
+      <c r="D5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6">
+        <v>28.06666666666667</v>
+      </c>
+      <c r="C6">
+        <v>18.28862998331659</v>
+      </c>
+      <c r="D6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7">
+        <v>16.23166666666667</v>
+      </c>
+      <c r="C7">
+        <v>7.690826786936935</v>
+      </c>
+      <c r="D7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8">
+        <v>27.10166666666667</v>
+      </c>
+      <c r="C8">
+        <v>22.22504210719671</v>
+      </c>
+      <c r="D8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9">
+        <v>11.51</v>
+      </c>
+      <c r="C9">
+        <v>7.301079372257227</v>
+      </c>
+      <c r="D9">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10">
+        <v>3.983333333333334</v>
+      </c>
+      <c r="C10">
+        <v>3.994389398477153</v>
+      </c>
+      <c r="D10">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11">
+        <v>25.54</v>
+      </c>
+      <c r="C11">
+        <v>19.87033869867346</v>
+      </c>
+      <c r="D11">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12">
+        <v>17.22166666666667</v>
+      </c>
+      <c r="C12">
+        <v>15.55391322679494</v>
+      </c>
+      <c r="D12">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13">
+        <v>32.38</v>
+      </c>
+      <c r="C13">
+        <v>30.10027375290796</v>
+      </c>
+      <c r="D13">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14">
+        <v>39.72333333333334</v>
+      </c>
+      <c r="C14">
+        <v>35.28562351251097</v>
+      </c>
+      <c r="D14">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15">
+        <v>42.07833333333333</v>
+      </c>
+      <c r="C15">
+        <v>33.11973455006346</v>
+      </c>
+      <c r="D15">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16">
+        <v>10.26833333333333</v>
+      </c>
+      <c r="C16">
+        <v>6.92675224522046</v>
+      </c>
+      <c r="D16">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17">
+        <v>42.98499999999999</v>
+      </c>
+      <c r="C17">
+        <v>41.07003420987132</v>
+      </c>
+      <c r="D17">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18">
+        <v>37.60333333333333</v>
+      </c>
+      <c r="C18">
+        <v>18.19036961325049</v>
+      </c>
+      <c r="D18">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19">
+        <v>38.35</v>
+      </c>
+      <c r="C19">
+        <v>33.34598806453334</v>
+      </c>
+      <c r="D19">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20">
+        <v>6.235</v>
+      </c>
+      <c r="C20">
+        <v>6.190126816148438</v>
+      </c>
+      <c r="D20">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -1113,30 +1240,30 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B2">
-        <v>24.2436170212766</v>
+        <v>23.57535714285714</v>
       </c>
       <c r="C2">
-        <v>24.59431450961716</v>
+        <v>24.17808519106701</v>
       </c>
       <c r="D2">
-        <v>47</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B3">
-        <v>25.11625</v>
+        <v>24.49526315789474</v>
       </c>
       <c r="C3">
-        <v>25.33856514309045</v>
+        <v>25.11074642638537</v>
       </c>
       <c r="D3">
-        <v>48</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>